<commit_message>
Ensure songs are consistent between XLSX and JSON
</commit_message>
<xml_diff>
--- a/data/Depeche Mode Songs.xlsx
+++ b/data/Depeche Mode Songs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lindanakasone/Documents/GitHub/playlist-visualized/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B788B460-A41D-FF44-8876-7EF5081C18C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC2E83F2-8262-104B-B0E0-00FF2048B8EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3080" yWindow="3120" windowWidth="36160" windowHeight="22780" xr2:uid="{FE581154-A771-454D-BC0C-F4CC813A6F29}"/>
   </bookViews>
@@ -871,19 +871,19 @@
     <t>Sea of Sin (Tonal Mix)</t>
   </si>
   <si>
-    <t>Survive (from the "Memento Mori" sessions)</t>
-  </si>
-  <si>
-    <t>Life 2.0 (from the "Memento Mori" sessions)</t>
-  </si>
-  <si>
-    <t>Give Yourself To Me (from the "Memento Mori" sessions)</t>
-  </si>
-  <si>
-    <t>In The End (from the "Memento Mori" sessions)</t>
-  </si>
-  <si>
     <t>Memento Mori: Mexico City</t>
+  </si>
+  <si>
+    <t>In The End (from the Memento Mori Sessions)</t>
+  </si>
+  <si>
+    <t>Give Yourself To Me (from the Memento Mori Sessions)</t>
+  </si>
+  <si>
+    <t>Life 2.0 (from the Memento Mori Sessions)</t>
+  </si>
+  <si>
+    <t>Survive (from the Memento Mori Sessions)</t>
   </si>
 </sst>
 </file>
@@ -5214,10 +5214,10 @@
     </row>
     <row r="247" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A247" t="s">
+        <v>286</v>
+      </c>
+      <c r="B247" t="s">
         <v>282</v>
-      </c>
-      <c r="B247" t="s">
-        <v>286</v>
       </c>
       <c r="C247">
         <v>2025</v>
@@ -5228,10 +5228,10 @@
     </row>
     <row r="248" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A248" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B248" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="C248">
         <v>2025</v>
@@ -5245,7 +5245,7 @@
         <v>284</v>
       </c>
       <c r="B249" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="C249">
         <v>2025</v>
@@ -5256,10 +5256,10 @@
     </row>
     <row r="250" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="B250" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="C250">
         <v>2025</v>

</xml_diff>

<commit_message>
completed the Xlsx and JSON associated with Depeche Mode songs
</commit_message>
<xml_diff>
--- a/data/Depeche Mode Songs.xlsx
+++ b/data/Depeche Mode Songs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lindanakasone/Documents/GitHub/playlist-visualized/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC2E83F2-8262-104B-B0E0-00FF2048B8EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77A5F825-5AB8-D04B-82EB-58EC51E79DC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3080" yWindow="3120" windowWidth="36160" windowHeight="22780" xr2:uid="{FE581154-A771-454D-BC0C-F4CC813A6F29}"/>
+    <workbookView xWindow="16320" yWindow="4460" windowWidth="36160" windowHeight="22780" xr2:uid="{FE581154-A771-454D-BC0C-F4CC813A6F29}"/>
   </bookViews>
   <sheets>
     <sheet name="Depeche Mode Songs" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="751" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="823" uniqueCount="311">
   <si>
     <t>Song</t>
   </si>
@@ -884,6 +884,78 @@
   </si>
   <si>
     <t>Survive (from the Memento Mori Sessions)</t>
+  </si>
+  <si>
+    <t>Intro (Live In Mexico City)</t>
+  </si>
+  <si>
+    <t>My Cosmos Is Mine (Live In Mexico City)</t>
+  </si>
+  <si>
+    <t>Wagging Tongue (Live In Mexico City)</t>
+  </si>
+  <si>
+    <t>Walking In My Shoes (Live In Mexico City)</t>
+  </si>
+  <si>
+    <t>It's No Good (Live In Mexico City)</t>
+  </si>
+  <si>
+    <t>Sister of Night (Live In Mexico City)</t>
+  </si>
+  <si>
+    <t>In Your Room (Live In Mexico City)</t>
+  </si>
+  <si>
+    <t>Everything Counts (Live In Mexico City)</t>
+  </si>
+  <si>
+    <t>Precious (Live In Mexico City)</t>
+  </si>
+  <si>
+    <t>Speak To Me (Live In Mexico City)</t>
+  </si>
+  <si>
+    <t>Home (Live In Mexico City)</t>
+  </si>
+  <si>
+    <t>Soul With Me (Live In Mexico City)</t>
+  </si>
+  <si>
+    <t>Ghosts Again (Live In Mexico City)</t>
+  </si>
+  <si>
+    <t>I Feel You (Live In Mexico City)</t>
+  </si>
+  <si>
+    <t>A Pain That I'm Used To (Live In Mexico City)</t>
+  </si>
+  <si>
+    <t>World In My Eyes (Live In Mexico City)</t>
+  </si>
+  <si>
+    <t>Wrong (Live In Mexico City)</t>
+  </si>
+  <si>
+    <t>Stripped (Live In Mexico City)</t>
+  </si>
+  <si>
+    <t>John The Revelator (Live In Mexico City)</t>
+  </si>
+  <si>
+    <t>Enjoy The Silence (Live In Mexico City)</t>
+  </si>
+  <si>
+    <t>Waiting For The Night (Live In Mexico City)</t>
+  </si>
+  <si>
+    <t>Just Can't Get Enough (Live In Mexico City)</t>
+  </si>
+  <si>
+    <t>Never Let Me Down Again (Live In Mexico City)</t>
+  </si>
+  <si>
+    <t>Personal Jesus (Live In Mexico City)</t>
   </si>
 </sst>
 </file>
@@ -1759,10 +1831,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE1C0B07-670E-FB45-A921-EAB11111294F}">
-  <dimension ref="A1:G250"/>
+  <dimension ref="A1:G274"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="37.83203125" customWidth="1"/>
+    <col min="2" max="2" width="33.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
@@ -5128,7 +5201,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="241" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
         <v>263</v>
       </c>
@@ -5142,7 +5215,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="242" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
         <v>264</v>
       </c>
@@ -5156,7 +5229,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="243" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A243" t="s">
         <v>265</v>
       </c>
@@ -5170,7 +5243,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="244" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A244" t="s">
         <v>266</v>
       </c>
@@ -5184,7 +5257,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="245" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A245" t="s">
         <v>267</v>
       </c>
@@ -5198,7 +5271,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="246" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A246" t="s">
         <v>268</v>
       </c>
@@ -5212,7 +5285,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="247" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A247" t="s">
         <v>286</v>
       </c>
@@ -5226,7 +5299,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="248" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A248" t="s">
         <v>285</v>
       </c>
@@ -5240,7 +5313,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="249" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A249" t="s">
         <v>284</v>
       </c>
@@ -5254,7 +5327,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="250" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
         <v>283</v>
       </c>
@@ -5266,6 +5339,270 @@
       </c>
       <c r="D250" t="s">
         <v>271</v>
+      </c>
+    </row>
+    <row r="251" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A251" t="s">
+        <v>287</v>
+      </c>
+      <c r="B251" t="s">
+        <v>282</v>
+      </c>
+      <c r="F251" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="252" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A252" t="s">
+        <v>288</v>
+      </c>
+      <c r="B252" t="s">
+        <v>282</v>
+      </c>
+      <c r="F252" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="253" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A253" t="s">
+        <v>289</v>
+      </c>
+      <c r="B253" t="s">
+        <v>282</v>
+      </c>
+      <c r="F253" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="254" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A254" t="s">
+        <v>290</v>
+      </c>
+      <c r="B254" t="s">
+        <v>282</v>
+      </c>
+      <c r="F254" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="255" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A255" t="s">
+        <v>291</v>
+      </c>
+      <c r="B255" t="s">
+        <v>282</v>
+      </c>
+      <c r="F255" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="256" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A256" t="s">
+        <v>292</v>
+      </c>
+      <c r="B256" t="s">
+        <v>282</v>
+      </c>
+      <c r="F256" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="257" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A257" t="s">
+        <v>293</v>
+      </c>
+      <c r="B257" t="s">
+        <v>282</v>
+      </c>
+      <c r="F257" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="258" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A258" t="s">
+        <v>294</v>
+      </c>
+      <c r="B258" t="s">
+        <v>282</v>
+      </c>
+      <c r="F258" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="259" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A259" t="s">
+        <v>295</v>
+      </c>
+      <c r="B259" t="s">
+        <v>282</v>
+      </c>
+      <c r="F259" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="260" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A260" t="s">
+        <v>296</v>
+      </c>
+      <c r="B260" t="s">
+        <v>282</v>
+      </c>
+      <c r="F260" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="261" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A261" t="s">
+        <v>297</v>
+      </c>
+      <c r="B261" t="s">
+        <v>282</v>
+      </c>
+      <c r="F261" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="262" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A262" t="s">
+        <v>298</v>
+      </c>
+      <c r="B262" t="s">
+        <v>282</v>
+      </c>
+      <c r="F262" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="263" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A263" t="s">
+        <v>299</v>
+      </c>
+      <c r="B263" t="s">
+        <v>282</v>
+      </c>
+      <c r="F263" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="264" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A264" t="s">
+        <v>300</v>
+      </c>
+      <c r="B264" t="s">
+        <v>282</v>
+      </c>
+      <c r="F264" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="265" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A265" t="s">
+        <v>301</v>
+      </c>
+      <c r="B265" t="s">
+        <v>282</v>
+      </c>
+      <c r="F265" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="266" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A266" t="s">
+        <v>302</v>
+      </c>
+      <c r="B266" t="s">
+        <v>282</v>
+      </c>
+      <c r="F266" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="267" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A267" t="s">
+        <v>303</v>
+      </c>
+      <c r="B267" t="s">
+        <v>282</v>
+      </c>
+      <c r="F267" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="268" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A268" t="s">
+        <v>304</v>
+      </c>
+      <c r="B268" t="s">
+        <v>282</v>
+      </c>
+      <c r="F268" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="269" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A269" t="s">
+        <v>305</v>
+      </c>
+      <c r="B269" t="s">
+        <v>282</v>
+      </c>
+      <c r="F269" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="270" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A270" t="s">
+        <v>306</v>
+      </c>
+      <c r="B270" t="s">
+        <v>282</v>
+      </c>
+      <c r="F270" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="271" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A271" t="s">
+        <v>307</v>
+      </c>
+      <c r="B271" t="s">
+        <v>282</v>
+      </c>
+      <c r="F271" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="272" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A272" t="s">
+        <v>308</v>
+      </c>
+      <c r="B272" t="s">
+        <v>282</v>
+      </c>
+      <c r="F272" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="273" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A273" t="s">
+        <v>309</v>
+      </c>
+      <c r="B273" t="s">
+        <v>282</v>
+      </c>
+      <c r="F273" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="274" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A274" t="s">
+        <v>310</v>
+      </c>
+      <c r="B274" t="s">
+        <v>282</v>
+      </c>
+      <c r="F274" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>